<commit_message>
al-imran corrections 191و 185
</commit_message>
<xml_diff>
--- a/verification_summary.xlsx
+++ b/verification_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E40"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1109,168 +1109,210 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>111</t>
+          <t>003</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>سورة 111</t>
+          <t>سورة 3</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>5431</v>
+        <v>1055764</v>
       </c>
       <c r="D33" t="n">
-        <v>8447</v>
+        <v>1673326</v>
       </c>
       <c r="E33" t="n">
-        <v>3016</v>
+        <v>617562</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>110</t>
+          <t>004</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>سورة 110</t>
+          <t>سورة 4</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>6123</v>
+        <v>1060245</v>
       </c>
       <c r="D34" t="n">
-        <v>9368</v>
+        <v>1706449</v>
       </c>
       <c r="E34" t="n">
-        <v>3245</v>
+        <v>646204</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>080</t>
+          <t>111</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>سورة 80</t>
+          <t>سورة 111</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>46973</v>
+        <v>5431</v>
       </c>
       <c r="D35" t="n">
-        <v>68652</v>
+        <v>8447</v>
       </c>
       <c r="E35" t="n">
-        <v>21679</v>
+        <v>3016</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>087</t>
+          <t>110</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>سورة 87</t>
+          <t>سورة 110</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>25500</v>
+        <v>6123</v>
       </c>
       <c r="D36" t="n">
-        <v>36391</v>
+        <v>9368</v>
       </c>
       <c r="E36" t="n">
-        <v>10891</v>
+        <v>3245</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>089</t>
+          <t>080</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>سورة 89</t>
+          <t>سورة 80</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>47933</v>
+        <v>46973</v>
       </c>
       <c r="D37" t="n">
-        <v>71615</v>
+        <v>68652</v>
       </c>
       <c r="E37" t="n">
-        <v>23682</v>
+        <v>21679</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>088</t>
+          <t>087</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>سورة 88</t>
+          <t>سورة 87</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>31098</v>
+        <v>25500</v>
       </c>
       <c r="D38" t="n">
-        <v>45729</v>
+        <v>36391</v>
       </c>
       <c r="E38" t="n">
-        <v>14631</v>
+        <v>10891</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>086</t>
+          <t>089</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>سورة 86</t>
+          <t>سورة 89</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>16572</v>
+        <v>47933</v>
       </c>
       <c r="D39" t="n">
-        <v>27797</v>
+        <v>71615</v>
       </c>
       <c r="E39" t="n">
-        <v>11225</v>
+        <v>23682</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
+          <t>088</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>سورة 88</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>31098</v>
+      </c>
+      <c r="D40" t="n">
+        <v>45729</v>
+      </c>
+      <c r="E40" t="n">
+        <v>14631</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>086</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>سورة 86</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>16572</v>
+      </c>
+      <c r="D41" t="n">
+        <v>27797</v>
+      </c>
+      <c r="E41" t="n">
+        <v>11225</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
           <t>081</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr">
+      <c r="B42" t="inlineStr">
         <is>
           <t>سورة 81</t>
         </is>
       </c>
-      <c r="C40" t="n">
+      <c r="C42" t="n">
         <v>40267</v>
       </c>
-      <c r="D40" t="n">
+      <c r="D42" t="n">
         <v>59707</v>
       </c>
-      <c r="E40" t="n">
+      <c r="E42" t="n">
         <v>19440</v>
       </c>
     </row>

</xml_diff>

<commit_message>
surah al-anfaal: correction 50 72
</commit_message>
<xml_diff>
--- a/verification_summary.xlsx
+++ b/verification_summary.xlsx
@@ -719,13 +719,13 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>375219</v>
+        <v>375580</v>
       </c>
       <c r="D14" t="n">
-        <v>599442</v>
+        <v>597162</v>
       </c>
       <c r="E14" t="n">
-        <v>224223</v>
+        <v>221582</v>
       </c>
     </row>
     <row r="15">
@@ -740,13 +740,13 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0</v>
+        <v>247323</v>
       </c>
       <c r="D15" t="n">
-        <v>0</v>
+        <v>402451</v>
       </c>
       <c r="E15" t="n">
-        <v>0</v>
+        <v>155128</v>
       </c>
     </row>
     <row r="16">

</xml_diff>

<commit_message>
surah yunus verses 30
</commit_message>
<xml_diff>
--- a/verification_summary.xlsx
+++ b/verification_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E51"/>
+  <dimension ref="A1:E53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -740,13 +740,13 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>724330</v>
+        <v>737716</v>
       </c>
       <c r="D15" t="n">
-        <v>1171491</v>
+        <v>1187765</v>
       </c>
       <c r="E15" t="n">
-        <v>447161</v>
+        <v>450049</v>
       </c>
     </row>
     <row r="16">
@@ -1046,463 +1046,505 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>095</t>
+          <t>059</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>سورة 95</t>
+          <t>سورة 59</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>10228</v>
+        <v>126461</v>
       </c>
       <c r="D30" t="n">
-        <v>17123</v>
+        <v>204801</v>
       </c>
       <c r="E30" t="n">
-        <v>6895</v>
+        <v>78340</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>094</t>
+          <t>095</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>سورة 94</t>
+          <t>سورة 95</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>12416</v>
+        <v>10228</v>
       </c>
       <c r="D31" t="n">
-        <v>16921</v>
+        <v>17123</v>
       </c>
       <c r="E31" t="n">
-        <v>4505</v>
+        <v>6895</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>093</t>
+          <t>094</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>سورة 93</t>
+          <t>سورة 94</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>12482</v>
+        <v>12416</v>
       </c>
       <c r="D32" t="n">
-        <v>18986</v>
+        <v>16921</v>
       </c>
       <c r="E32" t="n">
-        <v>6504</v>
+        <v>4505</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>058</t>
+          <t>093</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>سورة 58</t>
+          <t>سورة 93</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>0</v>
+        <v>12482</v>
       </c>
       <c r="D33" t="n">
-        <v>0</v>
+        <v>18986</v>
       </c>
       <c r="E33" t="n">
-        <v>0</v>
+        <v>6504</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>056</t>
+          <t>058</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>سورة 56</t>
+          <t>سورة 58</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>0</v>
+        <v>131237</v>
       </c>
       <c r="D34" t="n">
-        <v>0</v>
+        <v>213351</v>
       </c>
       <c r="E34" t="n">
-        <v>0</v>
+        <v>82114</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>005</t>
+          <t>056</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>سورة 5</t>
+          <t>سورة 56</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>824051</v>
+        <v>0</v>
       </c>
       <c r="D35" t="n">
-        <v>1342319</v>
+        <v>0</v>
       </c>
       <c r="E35" t="n">
-        <v>518268</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>002</t>
+          <t>005</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>سورة 2</t>
+          <t>سورة 5</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>1823935</v>
+        <v>824051</v>
       </c>
       <c r="D36" t="n">
-        <v>2916192</v>
+        <v>1342319</v>
       </c>
       <c r="E36" t="n">
-        <v>1092257</v>
+        <v>518268</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>104</t>
+          <t>002</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>سورة 104</t>
+          <t>سورة 2</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>5947</v>
+        <v>1823935</v>
       </c>
       <c r="D37" t="n">
-        <v>11245</v>
+        <v>2916192</v>
       </c>
       <c r="E37" t="n">
-        <v>5298</v>
+        <v>1092257</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>103</t>
+          <t>104</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>سورة 103</t>
+          <t>سورة 104</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>4740</v>
+        <v>5947</v>
       </c>
       <c r="D38" t="n">
-        <v>7972</v>
+        <v>11245</v>
       </c>
       <c r="E38" t="n">
-        <v>3232</v>
+        <v>5298</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>102</t>
+          <t>103</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>سورة 102</t>
+          <t>سورة 103</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>10365</v>
+        <v>4740</v>
       </c>
       <c r="D39" t="n">
-        <v>15267</v>
+        <v>7972</v>
       </c>
       <c r="E39" t="n">
-        <v>4902</v>
+        <v>3232</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>105</t>
+          <t>102</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>سورة 105</t>
+          <t>سورة 102</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>5470</v>
+        <v>10365</v>
       </c>
       <c r="D40" t="n">
-        <v>8775</v>
+        <v>15267</v>
       </c>
       <c r="E40" t="n">
-        <v>3305</v>
+        <v>4902</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>003</t>
+          <t>105</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>سورة 3</t>
+          <t>سورة 105</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>1055770</v>
+        <v>5470</v>
       </c>
       <c r="D41" t="n">
-        <v>1673992</v>
+        <v>8775</v>
       </c>
       <c r="E41" t="n">
-        <v>618222</v>
+        <v>3305</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>004</t>
+          <t>003</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>سورة 4</t>
+          <t>سورة 3</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>1116433</v>
+        <v>1055770</v>
       </c>
       <c r="D42" t="n">
-        <v>1798405</v>
+        <v>1673992</v>
       </c>
       <c r="E42" t="n">
-        <v>681972</v>
+        <v>618222</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>111</t>
+          <t>004</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>سورة 111</t>
+          <t>سورة 4</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>5431</v>
+        <v>1116433</v>
       </c>
       <c r="D43" t="n">
-        <v>8447</v>
+        <v>1798405</v>
       </c>
       <c r="E43" t="n">
-        <v>3016</v>
+        <v>681972</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>110</t>
+          <t>111</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>سورة 110</t>
+          <t>سورة 111</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>6123</v>
+        <v>5431</v>
       </c>
       <c r="D44" t="n">
-        <v>9368</v>
+        <v>8447</v>
       </c>
       <c r="E44" t="n">
-        <v>3245</v>
+        <v>3016</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>080</t>
+          <t>110</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>سورة 80</t>
+          <t>سورة 110</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>46973</v>
+        <v>6123</v>
       </c>
       <c r="D45" t="n">
-        <v>68652</v>
+        <v>9368</v>
       </c>
       <c r="E45" t="n">
-        <v>21679</v>
+        <v>3245</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>087</t>
+          <t>080</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>سورة 87</t>
+          <t>سورة 80</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>25500</v>
+        <v>46973</v>
       </c>
       <c r="D46" t="n">
-        <v>36391</v>
+        <v>68652</v>
       </c>
       <c r="E46" t="n">
-        <v>10891</v>
+        <v>21679</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>089</t>
+          <t>087</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>سورة 89</t>
+          <t>سورة 87</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>47933</v>
+        <v>25500</v>
       </c>
       <c r="D47" t="n">
-        <v>71615</v>
+        <v>36391</v>
       </c>
       <c r="E47" t="n">
-        <v>23682</v>
+        <v>10891</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>088</t>
+          <t>089</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>سورة 88</t>
+          <t>سورة 89</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>31098</v>
+        <v>47933</v>
       </c>
       <c r="D48" t="n">
-        <v>45729</v>
+        <v>71615</v>
       </c>
       <c r="E48" t="n">
-        <v>14631</v>
+        <v>23682</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>086</t>
+          <t>011</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>سورة 86</t>
+          <t>سورة 11</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>16572</v>
+        <v>0</v>
       </c>
       <c r="D49" t="n">
-        <v>27797</v>
+        <v>0</v>
       </c>
       <c r="E49" t="n">
-        <v>11225</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>081</t>
+          <t>088</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>سورة 81</t>
+          <t>سورة 88</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>40267</v>
+        <v>31098</v>
       </c>
       <c r="D50" t="n">
-        <v>59707</v>
+        <v>45729</v>
       </c>
       <c r="E50" t="n">
-        <v>19440</v>
+        <v>14631</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
+          <t>086</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>سورة 86</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>16572</v>
+      </c>
+      <c r="D51" t="n">
+        <v>27797</v>
+      </c>
+      <c r="E51" t="n">
+        <v>11225</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>081</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>سورة 81</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>40267</v>
+      </c>
+      <c r="D52" t="n">
+        <v>59707</v>
+      </c>
+      <c r="E52" t="n">
+        <v>19440</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
           <t>010</t>
         </is>
       </c>
-      <c r="B51" t="inlineStr">
+      <c r="B53" t="inlineStr">
         <is>
           <t>سورة 10</t>
         </is>
       </c>
-      <c r="C51" t="n">
-        <v>786</v>
-      </c>
-      <c r="D51" t="n">
-        <v>1553</v>
-      </c>
-      <c r="E51" t="n">
-        <v>767</v>
+      <c r="C53" t="n">
+        <v>52295</v>
+      </c>
+      <c r="D53" t="n">
+        <v>88327</v>
+      </c>
+      <c r="E53" t="n">
+        <v>36032</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
surah hud corrections 64
</commit_message>
<xml_diff>
--- a/verification_summary.xlsx
+++ b/verification_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E53"/>
+  <dimension ref="A1:E115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -458,1093 +458,2395 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>098</t>
+          <t>053</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>سورة 98</t>
+          <t>سورة 53</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>28085</v>
+        <v>106640</v>
       </c>
       <c r="D2" t="n">
-        <v>43441</v>
+        <v>166401</v>
       </c>
       <c r="E2" t="n">
-        <v>15356</v>
+        <v>59761</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>096</t>
+          <t>098</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>سورة 96</t>
+          <t>سورة 98</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>9571</v>
+        <v>28085</v>
       </c>
       <c r="D3" t="n">
-        <v>16252</v>
+        <v>43441</v>
       </c>
       <c r="E3" t="n">
-        <v>6681</v>
+        <v>15356</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>091</t>
+          <t>054</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>سورة 91</t>
+          <t>سورة 54</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>18941</v>
+        <v>118384</v>
       </c>
       <c r="D4" t="n">
-        <v>29116</v>
+        <v>178000</v>
       </c>
       <c r="E4" t="n">
-        <v>10175</v>
+        <v>59616</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>090</t>
+          <t>096</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>سورة 90</t>
+          <t>سورة 96</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>20308</v>
+        <v>9571</v>
       </c>
       <c r="D5" t="n">
-        <v>34633</v>
+        <v>16252</v>
       </c>
       <c r="E5" t="n">
-        <v>14325</v>
+        <v>6681</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>097</t>
+          <t>062</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>سورة 97</t>
+          <t>سورة 62</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>6711</v>
+        <v>59597</v>
       </c>
       <c r="D6" t="n">
-        <v>11025</v>
+        <v>90538</v>
       </c>
       <c r="E6" t="n">
-        <v>4314</v>
+        <v>30941</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>055</t>
+          <t>065</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>سورة 55</t>
+          <t>سورة 65</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>117677</v>
+        <v>89368</v>
       </c>
       <c r="D7" t="n">
-        <v>182612</v>
+        <v>136982</v>
       </c>
       <c r="E7" t="n">
-        <v>64935</v>
+        <v>47614</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>099</t>
+          <t>091</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>سورة 99</t>
+          <t>سورة 91</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>16589</v>
+        <v>18941</v>
       </c>
       <c r="D8" t="n">
-        <v>23384</v>
+        <v>29116</v>
       </c>
       <c r="E8" t="n">
-        <v>6795</v>
+        <v>10175</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>031</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>سورة 1</t>
+          <t>سورة 31</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>10145</v>
+        <v>155322</v>
       </c>
       <c r="D9" t="n">
-        <v>16281</v>
+        <v>242378</v>
       </c>
       <c r="E9" t="n">
-        <v>6136</v>
+        <v>87056</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>109</t>
+          <t>036</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>سورة 109</t>
+          <t>سورة 36</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>3828</v>
+        <v>217025</v>
       </c>
       <c r="D10" t="n">
-        <v>8390</v>
+        <v>344953</v>
       </c>
       <c r="E10" t="n">
-        <v>4562</v>
+        <v>127928</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>006</t>
+          <t>038</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>سورة 6</t>
+          <t>سورة 38</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>933118</v>
+        <v>227718</v>
       </c>
       <c r="D11" t="n">
-        <v>1454355</v>
+        <v>359151</v>
       </c>
       <c r="E11" t="n">
-        <v>521237</v>
+        <v>131433</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>090</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>سورة 100</t>
+          <t>سورة 90</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>13357</v>
+        <v>20309</v>
       </c>
       <c r="D12" t="n">
-        <v>19431</v>
+        <v>34744</v>
       </c>
       <c r="E12" t="n">
-        <v>6074</v>
+        <v>14435</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>107</t>
+          <t>064</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>سورة 107</t>
+          <t>سورة 64</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>9206</v>
+        <v>78577</v>
       </c>
       <c r="D13" t="n">
-        <v>13645</v>
+        <v>121321</v>
       </c>
       <c r="E13" t="n">
-        <v>4439</v>
+        <v>42744</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>008</t>
+          <t>063</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>سورة 8</t>
+          <t>سورة 63</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>375580</v>
+        <v>53288</v>
       </c>
       <c r="D14" t="n">
-        <v>597162</v>
+        <v>86067</v>
       </c>
       <c r="E14" t="n">
-        <v>221582</v>
+        <v>32779</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>009</t>
+          <t>097</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>سورة 9</t>
+          <t>سورة 97</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>737716</v>
+        <v>6711</v>
       </c>
       <c r="D15" t="n">
-        <v>1187765</v>
+        <v>11025</v>
       </c>
       <c r="E15" t="n">
-        <v>450049</v>
+        <v>4314</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>106</t>
+          <t>055</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>سورة 106</t>
+          <t>سورة 55</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>5656</v>
+        <v>126514</v>
       </c>
       <c r="D16" t="n">
-        <v>8344</v>
+        <v>198518</v>
       </c>
       <c r="E16" t="n">
-        <v>2688</v>
+        <v>72004</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>101</t>
+          <t>052</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>سورة 101</t>
+          <t>سورة 52</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>9883</v>
+        <v>93393</v>
       </c>
       <c r="D17" t="n">
-        <v>16934</v>
+        <v>144964</v>
       </c>
       <c r="E17" t="n">
-        <v>7051</v>
+        <v>51571</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>007</t>
+          <t>099</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>سورة 7</t>
+          <t>سورة 99</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>1053563</v>
+        <v>16589</v>
       </c>
       <c r="D18" t="n">
-        <v>1663572</v>
+        <v>23384</v>
       </c>
       <c r="E18" t="n">
-        <v>610009</v>
+        <v>6795</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>108</t>
+          <t>039</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>سورة 108</t>
+          <t>سورة 39</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>2753</v>
+        <v>364749</v>
       </c>
       <c r="D19" t="n">
-        <v>4670</v>
+        <v>558075</v>
       </c>
       <c r="E19" t="n">
-        <v>1917</v>
+        <v>193326</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>112</t>
+          <t>037</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>سورة 112</t>
+          <t>سورة 37</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>1002</v>
+        <v>259584</v>
       </c>
       <c r="D20" t="n">
-        <v>2858</v>
+        <v>421472</v>
       </c>
       <c r="E20" t="n">
-        <v>1856</v>
+        <v>161888</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>114</t>
+          <t>030</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>سورة 114</t>
+          <t>سورة 30</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>4901</v>
+        <v>268137</v>
       </c>
       <c r="D21" t="n">
-        <v>9118</v>
+        <v>405129</v>
       </c>
       <c r="E21" t="n">
-        <v>4217</v>
+        <v>136992</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>113</t>
+          <t>001</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>سورة 113</t>
+          <t>سورة 1</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>8675</v>
+        <v>10145</v>
       </c>
       <c r="D22" t="n">
-        <v>11985</v>
+        <v>16281</v>
       </c>
       <c r="E22" t="n">
-        <v>3310</v>
+        <v>6136</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>084</t>
+          <t>109</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>سورة 84</t>
+          <t>سورة 109</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>32937</v>
+        <v>3828</v>
       </c>
       <c r="D23" t="n">
-        <v>51519</v>
+        <v>8390</v>
       </c>
       <c r="E23" t="n">
-        <v>18582</v>
+        <v>4562</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>083</t>
+          <t>006</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>سورة 83</t>
+          <t>سورة 6</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>56682</v>
+        <v>933124</v>
       </c>
       <c r="D24" t="n">
-        <v>88370</v>
+        <v>1455021</v>
       </c>
       <c r="E24" t="n">
-        <v>31688</v>
+        <v>521897</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>079</t>
+          <t>100</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>سورة 79</t>
+          <t>سورة 100</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>59787</v>
+        <v>13357</v>
       </c>
       <c r="D25" t="n">
-        <v>92348</v>
+        <v>19431</v>
       </c>
       <c r="E25" t="n">
-        <v>32561</v>
+        <v>6074</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>078</t>
+          <t>107</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>سورة 78</t>
+          <t>سورة 107</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>53022</v>
+        <v>9206</v>
       </c>
       <c r="D26" t="n">
-        <v>89785</v>
+        <v>13645</v>
       </c>
       <c r="E26" t="n">
-        <v>36763</v>
+        <v>4439</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>082</t>
+          <t>008</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>سورة 82</t>
+          <t>سورة 8</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>26245</v>
+        <v>375581</v>
       </c>
       <c r="D27" t="n">
-        <v>40524</v>
+        <v>597273</v>
       </c>
       <c r="E27" t="n">
-        <v>14279</v>
+        <v>221692</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>085</t>
+          <t>009</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>سورة 85</t>
+          <t>سورة 9</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>32843</v>
+        <v>737716</v>
       </c>
       <c r="D28" t="n">
-        <v>50573</v>
+        <v>1187765</v>
       </c>
       <c r="E28" t="n">
-        <v>17730</v>
+        <v>450049</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>092</t>
+          <t>106</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>سورة 92</t>
+          <t>سورة 106</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>28806</v>
+        <v>5656</v>
       </c>
       <c r="D29" t="n">
-        <v>41746</v>
+        <v>8344</v>
       </c>
       <c r="E29" t="n">
-        <v>12940</v>
+        <v>2688</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>059</t>
+          <t>101</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>سورة 59</t>
+          <t>سورة 101</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>126461</v>
+        <v>9883</v>
       </c>
       <c r="D30" t="n">
-        <v>204801</v>
+        <v>16934</v>
       </c>
       <c r="E30" t="n">
-        <v>78340</v>
+        <v>7051</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>095</t>
+          <t>007</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>سورة 95</t>
+          <t>سورة 7</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>10228</v>
+        <v>1053576</v>
       </c>
       <c r="D31" t="n">
-        <v>17123</v>
+        <v>1665015</v>
       </c>
       <c r="E31" t="n">
-        <v>6895</v>
+        <v>611439</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>094</t>
+          <t>108</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>سورة 94</t>
+          <t>سورة 108</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>12416</v>
+        <v>2753</v>
       </c>
       <c r="D32" t="n">
-        <v>16921</v>
+        <v>4670</v>
       </c>
       <c r="E32" t="n">
-        <v>4505</v>
+        <v>1917</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>093</t>
+          <t>112</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>سورة 93</t>
+          <t>سورة 112</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>12482</v>
+        <v>1002</v>
       </c>
       <c r="D33" t="n">
-        <v>18986</v>
+        <v>2858</v>
       </c>
       <c r="E33" t="n">
-        <v>6504</v>
+        <v>1856</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>058</t>
+          <t>114</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>سورة 58</t>
+          <t>سورة 114</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>131237</v>
+        <v>4901</v>
       </c>
       <c r="D34" t="n">
-        <v>213351</v>
+        <v>9118</v>
       </c>
       <c r="E34" t="n">
-        <v>82114</v>
+        <v>4217</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>056</t>
+          <t>113</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>سورة 56</t>
+          <t>سورة 113</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>0</v>
+        <v>8675</v>
       </c>
       <c r="D35" t="n">
-        <v>0</v>
+        <v>11985</v>
       </c>
       <c r="E35" t="n">
-        <v>0</v>
+        <v>3310</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>005</t>
+          <t>012</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>سورة 5</t>
+          <t>سورة 12</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>824051</v>
+        <v>496610</v>
       </c>
       <c r="D36" t="n">
-        <v>1342319</v>
+        <v>818466</v>
       </c>
       <c r="E36" t="n">
-        <v>518268</v>
+        <v>321856</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>002</t>
+          <t>015</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>سورة 2</t>
+          <t>سورة 15</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>1823935</v>
+        <v>179659</v>
       </c>
       <c r="D37" t="n">
-        <v>2916192</v>
+        <v>303936</v>
       </c>
       <c r="E37" t="n">
-        <v>1092257</v>
+        <v>124277</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>104</t>
+          <t>023</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>سورة 104</t>
+          <t>سورة 23</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>5947</v>
+        <v>343106</v>
       </c>
       <c r="D38" t="n">
-        <v>11245</v>
+        <v>523833</v>
       </c>
       <c r="E38" t="n">
-        <v>5298</v>
+        <v>180727</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>103</t>
+          <t>024</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>سورة 103</t>
+          <t>سورة 24</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>4740</v>
+        <v>413694</v>
       </c>
       <c r="D39" t="n">
-        <v>7972</v>
+        <v>635921</v>
       </c>
       <c r="E39" t="n">
-        <v>3232</v>
+        <v>222227</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>102</t>
+          <t>084</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>سورة 102</t>
+          <t>سورة 84</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>10365</v>
+        <v>32936</v>
       </c>
       <c r="D40" t="n">
-        <v>15267</v>
+        <v>51408</v>
       </c>
       <c r="E40" t="n">
-        <v>4902</v>
+        <v>18472</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>105</t>
+          <t>070</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>سورة 105</t>
+          <t>سورة 70</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>5470</v>
+        <v>70490</v>
       </c>
       <c r="D41" t="n">
-        <v>8775</v>
+        <v>107786</v>
       </c>
       <c r="E41" t="n">
-        <v>3305</v>
+        <v>37296</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>003</t>
+          <t>048</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>سورة 3</t>
+          <t>سورة 48</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>1055770</v>
+        <v>181885</v>
       </c>
       <c r="D42" t="n">
-        <v>1673992</v>
+        <v>282023</v>
       </c>
       <c r="E42" t="n">
-        <v>618222</v>
+        <v>100138</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>004</t>
+          <t>077</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>سورة 4</t>
+          <t>سورة 77</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>1116433</v>
+        <v>71704</v>
       </c>
       <c r="D43" t="n">
-        <v>1798405</v>
+        <v>104802</v>
       </c>
       <c r="E43" t="n">
-        <v>681972</v>
+        <v>33098</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>111</t>
+          <t>083</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>سورة 111</t>
+          <t>سورة 83</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>5431</v>
+        <v>56682</v>
       </c>
       <c r="D44" t="n">
-        <v>8447</v>
+        <v>88370</v>
       </c>
       <c r="E44" t="n">
-        <v>3016</v>
+        <v>31688</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>110</t>
+          <t>041</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>سورة 110</t>
+          <t>سورة 41</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>6123</v>
+        <v>236367</v>
       </c>
       <c r="D45" t="n">
-        <v>9368</v>
+        <v>377290</v>
       </c>
       <c r="E45" t="n">
-        <v>3245</v>
+        <v>140923</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>080</t>
+          <t>079</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>سورة 80</t>
+          <t>سورة 79</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>46973</v>
+        <v>59787</v>
       </c>
       <c r="D46" t="n">
-        <v>68652</v>
+        <v>92348</v>
       </c>
       <c r="E46" t="n">
-        <v>21679</v>
+        <v>32561</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>087</t>
+          <t>046</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>سورة 87</t>
+          <t>سورة 46</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>25500</v>
+        <v>191842</v>
       </c>
       <c r="D47" t="n">
-        <v>36391</v>
+        <v>303283</v>
       </c>
       <c r="E47" t="n">
-        <v>10891</v>
+        <v>111441</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>089</t>
+          <t>025</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>سورة 89</t>
+          <t>سورة 25</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>47933</v>
+        <v>292108</v>
       </c>
       <c r="D48" t="n">
-        <v>71615</v>
+        <v>455117</v>
       </c>
       <c r="E48" t="n">
-        <v>23682</v>
+        <v>163009</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>011</t>
+          <t>022</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>سورة 11</t>
+          <t>سورة 22</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>0</v>
+        <v>364508</v>
       </c>
       <c r="D49" t="n">
-        <v>0</v>
+        <v>575624</v>
       </c>
       <c r="E49" t="n">
-        <v>0</v>
+        <v>211116</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>088</t>
+          <t>014</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>سورة 88</t>
+          <t>سورة 14</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>31098</v>
+        <v>263454</v>
       </c>
       <c r="D50" t="n">
-        <v>45729</v>
+        <v>407962</v>
       </c>
       <c r="E50" t="n">
-        <v>14631</v>
+        <v>144508</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>086</t>
+          <t>013</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>سورة 86</t>
+          <t>سورة 13</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>16572</v>
+        <v>238765</v>
       </c>
       <c r="D51" t="n">
-        <v>27797</v>
+        <v>381844</v>
       </c>
       <c r="E51" t="n">
-        <v>11225</v>
+        <v>143079</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>081</t>
+          <t>078</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>سورة 81</t>
+          <t>سورة 78</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>40267</v>
+        <v>53023</v>
       </c>
       <c r="D52" t="n">
-        <v>59707</v>
+        <v>89896</v>
       </c>
       <c r="E52" t="n">
-        <v>19440</v>
+        <v>36873</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
+          <t>047</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>سورة 47</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>180204</v>
+      </c>
+      <c r="D53" t="n">
+        <v>277718</v>
+      </c>
+      <c r="E53" t="n">
+        <v>97514</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>040</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>سورة 40</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>360481</v>
+      </c>
+      <c r="D54" t="n">
+        <v>570750</v>
+      </c>
+      <c r="E54" t="n">
+        <v>210269</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>049</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>سورة 49</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>101318</v>
+      </c>
+      <c r="D55" t="n">
+        <v>166033</v>
+      </c>
+      <c r="E55" t="n">
+        <v>64715</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>082</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>سورة 82</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>26245</v>
+      </c>
+      <c r="D56" t="n">
+        <v>40524</v>
+      </c>
+      <c r="E56" t="n">
+        <v>14279</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>076</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>سورة 76</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>73479</v>
+      </c>
+      <c r="D57" t="n">
+        <v>119000</v>
+      </c>
+      <c r="E57" t="n">
+        <v>45521</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>071</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>سورة 71</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>75292</v>
+      </c>
+      <c r="D58" t="n">
+        <v>117860</v>
+      </c>
+      <c r="E58" t="n">
+        <v>42568</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>085</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>سورة 85</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>32843</v>
+      </c>
+      <c r="D59" t="n">
+        <v>50573</v>
+      </c>
+      <c r="E59" t="n">
+        <v>17730</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>035</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>سورة 35</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>244447</v>
+      </c>
+      <c r="D60" t="n">
+        <v>375276</v>
+      </c>
+      <c r="E60" t="n">
+        <v>130829</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>032</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>سورة 32</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>110414</v>
+      </c>
+      <c r="D61" t="n">
+        <v>175850</v>
+      </c>
+      <c r="E61" t="n">
+        <v>65436</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>057</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>سورة 57</t>
+        </is>
+      </c>
+      <c r="C62" t="n">
+        <v>188928</v>
+      </c>
+      <c r="D62" t="n">
+        <v>287862</v>
+      </c>
+      <c r="E62" t="n">
+        <v>98934</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>068</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>سورة 68</t>
+        </is>
+      </c>
+      <c r="C63" t="n">
+        <v>90803</v>
+      </c>
+      <c r="D63" t="n">
+        <v>142935</v>
+      </c>
+      <c r="E63" t="n">
+        <v>52132</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>050</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>سورة 50</t>
+        </is>
+      </c>
+      <c r="C64" t="n">
+        <v>106854</v>
+      </c>
+      <c r="D64" t="n">
+        <v>166926</v>
+      </c>
+      <c r="E64" t="n">
+        <v>60072</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>066</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>سورة 66</t>
+        </is>
+      </c>
+      <c r="C65" t="n">
+        <v>85578</v>
+      </c>
+      <c r="D65" t="n">
+        <v>128504</v>
+      </c>
+      <c r="E65" t="n">
+        <v>42926</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>092</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>سورة 92</t>
+        </is>
+      </c>
+      <c r="C66" t="n">
+        <v>28806</v>
+      </c>
+      <c r="D66" t="n">
+        <v>41746</v>
+      </c>
+      <c r="E66" t="n">
+        <v>12940</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>059</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>سورة 59</t>
+        </is>
+      </c>
+      <c r="C67" t="n">
+        <v>126458</v>
+      </c>
+      <c r="D67" t="n">
+        <v>204468</v>
+      </c>
+      <c r="E67" t="n">
+        <v>78010</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>095</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>سورة 95</t>
+        </is>
+      </c>
+      <c r="C68" t="n">
+        <v>10228</v>
+      </c>
+      <c r="D68" t="n">
+        <v>17123</v>
+      </c>
+      <c r="E68" t="n">
+        <v>6895</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>061</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>سورة 61</t>
+        </is>
+      </c>
+      <c r="C69" t="n">
+        <v>61731</v>
+      </c>
+      <c r="D69" t="n">
+        <v>98696</v>
+      </c>
+      <c r="E69" t="n">
+        <v>36965</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>033</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>سورة 33</t>
+        </is>
+      </c>
+      <c r="C70" t="n">
+        <v>377184</v>
+      </c>
+      <c r="D70" t="n">
+        <v>619650</v>
+      </c>
+      <c r="E70" t="n">
+        <v>242466</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>034</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>سورة 34</t>
+        </is>
+      </c>
+      <c r="C71" t="n">
+        <v>254104</v>
+      </c>
+      <c r="D71" t="n">
+        <v>404044</v>
+      </c>
+      <c r="E71" t="n">
+        <v>149940</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>060</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>سورة 60</t>
+        </is>
+      </c>
+      <c r="C72" t="n">
+        <v>98862</v>
+      </c>
+      <c r="D72" t="n">
+        <v>163172</v>
+      </c>
+      <c r="E72" t="n">
+        <v>64310</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>094</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>سورة 94</t>
+        </is>
+      </c>
+      <c r="C73" t="n">
+        <v>12416</v>
+      </c>
+      <c r="D73" t="n">
+        <v>16921</v>
+      </c>
+      <c r="E73" t="n">
+        <v>4505</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>093</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>سورة 93</t>
+        </is>
+      </c>
+      <c r="C74" t="n">
+        <v>12482</v>
+      </c>
+      <c r="D74" t="n">
+        <v>18986</v>
+      </c>
+      <c r="E74" t="n">
+        <v>6504</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>067</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>سورة 67</t>
+        </is>
+      </c>
+      <c r="C75" t="n">
+        <v>102214</v>
+      </c>
+      <c r="D75" t="n">
+        <v>156456</v>
+      </c>
+      <c r="E75" t="n">
+        <v>54242</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>058</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>سورة 58</t>
+        </is>
+      </c>
+      <c r="C76" t="n">
+        <v>131236</v>
+      </c>
+      <c r="D76" t="n">
+        <v>213240</v>
+      </c>
+      <c r="E76" t="n">
+        <v>82004</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>051</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>سورة 51</t>
+        </is>
+      </c>
+      <c r="C77" t="n">
+        <v>116544</v>
+      </c>
+      <c r="D77" t="n">
+        <v>179352</v>
+      </c>
+      <c r="E77" t="n">
+        <v>62808</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>056</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>سورة 56</t>
+        </is>
+      </c>
+      <c r="C78" t="n">
+        <v>124148</v>
+      </c>
+      <c r="D78" t="n">
+        <v>196271</v>
+      </c>
+      <c r="E78" t="n">
+        <v>72123</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>069</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>سورة 69</t>
+        </is>
+      </c>
+      <c r="C79" t="n">
+        <v>84012</v>
+      </c>
+      <c r="D79" t="n">
+        <v>128119</v>
+      </c>
+      <c r="E79" t="n">
+        <v>44107</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>005</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>سورة 5</t>
+        </is>
+      </c>
+      <c r="C80" t="n">
+        <v>824052</v>
+      </c>
+      <c r="D80" t="n">
+        <v>1342430</v>
+      </c>
+      <c r="E80" t="n">
+        <v>518378</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>002</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>سورة 2</t>
+        </is>
+      </c>
+      <c r="C81" t="n">
+        <v>1823934</v>
+      </c>
+      <c r="D81" t="n">
+        <v>2916081</v>
+      </c>
+      <c r="E81" t="n">
+        <v>1092147</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>104</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>سورة 104</t>
+        </is>
+      </c>
+      <c r="C82" t="n">
+        <v>5947</v>
+      </c>
+      <c r="D82" t="n">
+        <v>11245</v>
+      </c>
+      <c r="E82" t="n">
+        <v>5298</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>103</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>سورة 103</t>
+        </is>
+      </c>
+      <c r="C83" t="n">
+        <v>4740</v>
+      </c>
+      <c r="D83" t="n">
+        <v>7972</v>
+      </c>
+      <c r="E83" t="n">
+        <v>3232</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>102</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>سورة 102</t>
+        </is>
+      </c>
+      <c r="C84" t="n">
+        <v>10365</v>
+      </c>
+      <c r="D84" t="n">
+        <v>15267</v>
+      </c>
+      <c r="E84" t="n">
+        <v>4902</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>105</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>سورة 105</t>
+        </is>
+      </c>
+      <c r="C85" t="n">
+        <v>5470</v>
+      </c>
+      <c r="D85" t="n">
+        <v>8775</v>
+      </c>
+      <c r="E85" t="n">
+        <v>3305</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>003</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>سورة 3</t>
+        </is>
+      </c>
+      <c r="C86" t="n">
+        <v>1055770</v>
+      </c>
+      <c r="D86" t="n">
+        <v>1673992</v>
+      </c>
+      <c r="E86" t="n">
+        <v>618222</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>004</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>سورة 4</t>
+        </is>
+      </c>
+      <c r="C87" t="n">
+        <v>1116432</v>
+      </c>
+      <c r="D87" t="n">
+        <v>1798294</v>
+      </c>
+      <c r="E87" t="n">
+        <v>681862</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>سورة 111</t>
+        </is>
+      </c>
+      <c r="C88" t="n">
+        <v>5431</v>
+      </c>
+      <c r="D88" t="n">
+        <v>8447</v>
+      </c>
+      <c r="E88" t="n">
+        <v>3016</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>110</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>سورة 110</t>
+        </is>
+      </c>
+      <c r="C89" t="n">
+        <v>6123</v>
+      </c>
+      <c r="D89" t="n">
+        <v>9368</v>
+      </c>
+      <c r="E89" t="n">
+        <v>3245</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>074</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>سورة 74</t>
+        </is>
+      </c>
+      <c r="C90" t="n">
+        <v>86563</v>
+      </c>
+      <c r="D90" t="n">
+        <v>128591</v>
+      </c>
+      <c r="E90" t="n">
+        <v>42028</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>080</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>سورة 80</t>
+        </is>
+      </c>
+      <c r="C91" t="n">
+        <v>46973</v>
+      </c>
+      <c r="D91" t="n">
+        <v>68652</v>
+      </c>
+      <c r="E91" t="n">
+        <v>21679</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>087</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>سورة 87</t>
+        </is>
+      </c>
+      <c r="C92" t="n">
+        <v>25500</v>
+      </c>
+      <c r="D92" t="n">
+        <v>36391</v>
+      </c>
+      <c r="E92" t="n">
+        <v>10891</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>073</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>سورة 73</t>
+        </is>
+      </c>
+      <c r="C93" t="n">
+        <v>67054</v>
+      </c>
+      <c r="D93" t="n">
+        <v>102874</v>
+      </c>
+      <c r="E93" t="n">
+        <v>35820</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>045</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>سورة 45</t>
+        </is>
+      </c>
+      <c r="C94" t="n">
+        <v>153278</v>
+      </c>
+      <c r="D94" t="n">
+        <v>236193</v>
+      </c>
+      <c r="E94" t="n">
+        <v>82915</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>089</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>سورة 89</t>
+        </is>
+      </c>
+      <c r="C95" t="n">
+        <v>47933</v>
+      </c>
+      <c r="D95" t="n">
+        <v>71615</v>
+      </c>
+      <c r="E95" t="n">
+        <v>23682</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>042</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>سورة 42</t>
+        </is>
+      </c>
+      <c r="C96" t="n">
+        <v>244353</v>
+      </c>
+      <c r="D96" t="n">
+        <v>382173</v>
+      </c>
+      <c r="E96" t="n">
+        <v>137820</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>016</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>سورة 16</t>
+        </is>
+      </c>
+      <c r="C97" t="n">
+        <v>557340</v>
+      </c>
+      <c r="D97" t="n">
+        <v>871332</v>
+      </c>
+      <c r="E97" t="n">
+        <v>313992</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>029</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>سورة 29</t>
+        </is>
+      </c>
+      <c r="C98" t="n">
+        <v>273996</v>
+      </c>
+      <c r="D98" t="n">
+        <v>455592</v>
+      </c>
+      <c r="E98" t="n">
+        <v>181596</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>011</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>سورة 11</t>
+        </is>
+      </c>
+      <c r="C99" t="n">
+        <v>537425</v>
+      </c>
+      <c r="D99" t="n">
+        <v>869436</v>
+      </c>
+      <c r="E99" t="n">
+        <v>332011</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>027</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>سورة 27</t>
+        </is>
+      </c>
+      <c r="C100" t="n">
+        <v>334206</v>
+      </c>
+      <c r="D100" t="n">
+        <v>532827</v>
+      </c>
+      <c r="E100" t="n">
+        <v>198621</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>018</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>سورة 18</t>
+        </is>
+      </c>
+      <c r="C101" t="n">
+        <v>495283</v>
+      </c>
+      <c r="D101" t="n">
+        <v>765360</v>
+      </c>
+      <c r="E101" t="n">
+        <v>270077</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>020</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>سورة 20</t>
+        </is>
+      </c>
+      <c r="C102" t="n">
+        <v>387551</v>
+      </c>
+      <c r="D102" t="n">
+        <v>608808</v>
+      </c>
+      <c r="E102" t="n">
+        <v>221257</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>088</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>سورة 88</t>
+        </is>
+      </c>
+      <c r="C103" t="n">
+        <v>31098</v>
+      </c>
+      <c r="D103" t="n">
+        <v>45729</v>
+      </c>
+      <c r="E103" t="n">
+        <v>14631</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>043</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>سورة 43</t>
+        </is>
+      </c>
+      <c r="C104" t="n">
+        <v>253805</v>
+      </c>
+      <c r="D104" t="n">
+        <v>399473</v>
+      </c>
+      <c r="E104" t="n">
+        <v>145668</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>044</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>سورة 44</t>
+        </is>
+      </c>
+      <c r="C105" t="n">
+        <v>95877</v>
+      </c>
+      <c r="D105" t="n">
+        <v>157791</v>
+      </c>
+      <c r="E105" t="n">
+        <v>61914</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>072</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>سورة 72</t>
+        </is>
+      </c>
+      <c r="C106" t="n">
+        <v>66493</v>
+      </c>
+      <c r="D106" t="n">
+        <v>116808</v>
+      </c>
+      <c r="E106" t="n">
+        <v>50315</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>086</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>سورة 86</t>
+        </is>
+      </c>
+      <c r="C107" t="n">
+        <v>16572</v>
+      </c>
+      <c r="D107" t="n">
+        <v>27797</v>
+      </c>
+      <c r="E107" t="n">
+        <v>11225</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>081</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>سورة 81</t>
+        </is>
+      </c>
+      <c r="C108" t="n">
+        <v>40267</v>
+      </c>
+      <c r="D108" t="n">
+        <v>59707</v>
+      </c>
+      <c r="E108" t="n">
+        <v>19440</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>075</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>سورة 75</t>
+        </is>
+      </c>
+      <c r="C109" t="n">
+        <v>48992</v>
+      </c>
+      <c r="D109" t="n">
+        <v>76987</v>
+      </c>
+      <c r="E109" t="n">
+        <v>27995</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>021</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>سورة 21</t>
+        </is>
+      </c>
+      <c r="C110" t="n">
+        <v>351038</v>
+      </c>
+      <c r="D110" t="n">
+        <v>559422</v>
+      </c>
+      <c r="E110" t="n">
+        <v>208384</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>026</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>سورة 26</t>
+        </is>
+      </c>
+      <c r="C111" t="n">
+        <v>391847</v>
+      </c>
+      <c r="D111" t="n">
+        <v>631520</v>
+      </c>
+      <c r="E111" t="n">
+        <v>239673</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>019</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>سورة 19</t>
+        </is>
+      </c>
+      <c r="C112" t="n">
+        <v>280985</v>
+      </c>
+      <c r="D112" t="n">
+        <v>444369</v>
+      </c>
+      <c r="E112" t="n">
+        <v>163384</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
           <t>010</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr">
+      <c r="B113" t="inlineStr">
         <is>
           <t>سورة 10</t>
         </is>
       </c>
-      <c r="C53" t="n">
-        <v>52295</v>
-      </c>
-      <c r="D53" t="n">
-        <v>88327</v>
-      </c>
-      <c r="E53" t="n">
-        <v>36032</v>
+      <c r="C113" t="n">
+        <v>535685</v>
+      </c>
+      <c r="D113" t="n">
+        <v>858951</v>
+      </c>
+      <c r="E113" t="n">
+        <v>323266</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>017</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>سورة 17</t>
+        </is>
+      </c>
+      <c r="C114" t="n">
+        <v>472754</v>
+      </c>
+      <c r="D114" t="n">
+        <v>753055</v>
+      </c>
+      <c r="E114" t="n">
+        <v>280301</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>028</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>سورة 28</t>
+        </is>
+      </c>
+      <c r="C115" t="n">
+        <v>399092</v>
+      </c>
+      <c r="D115" t="n">
+        <v>645325</v>
+      </c>
+      <c r="E115" t="n">
+        <v>246233</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
surah hud corrections 109
</commit_message>
<xml_diff>
--- a/verification_summary.xlsx
+++ b/verification_summary.xlsx
@@ -467,13 +467,13 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>106640</v>
+        <v>106630</v>
       </c>
       <c r="D2" t="n">
-        <v>166401</v>
+        <v>166390</v>
       </c>
       <c r="E2" t="n">
-        <v>59761</v>
+        <v>59760</v>
       </c>
     </row>
     <row r="3">
@@ -614,13 +614,13 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>155322</v>
+        <v>155320</v>
       </c>
       <c r="D9" t="n">
-        <v>242378</v>
+        <v>242156</v>
       </c>
       <c r="E9" t="n">
-        <v>87056</v>
+        <v>86836</v>
       </c>
     </row>
     <row r="10">
@@ -824,13 +824,13 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>364749</v>
+        <v>364747</v>
       </c>
       <c r="D19" t="n">
-        <v>558075</v>
+        <v>557853</v>
       </c>
       <c r="E19" t="n">
-        <v>193326</v>
+        <v>193106</v>
       </c>
     </row>
     <row r="20">
@@ -845,13 +845,13 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>259584</v>
+        <v>259583</v>
       </c>
       <c r="D20" t="n">
-        <v>421472</v>
+        <v>421361</v>
       </c>
       <c r="E20" t="n">
-        <v>161888</v>
+        <v>161778</v>
       </c>
     </row>
     <row r="21">
@@ -866,13 +866,13 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>268137</v>
+        <v>268136</v>
       </c>
       <c r="D21" t="n">
-        <v>405129</v>
+        <v>405018</v>
       </c>
       <c r="E21" t="n">
-        <v>136992</v>
+        <v>136882</v>
       </c>
     </row>
     <row r="22">
@@ -1013,13 +1013,13 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>737716</v>
+        <v>737713</v>
       </c>
       <c r="D28" t="n">
-        <v>1187765</v>
+        <v>1187432</v>
       </c>
       <c r="E28" t="n">
-        <v>450049</v>
+        <v>449719</v>
       </c>
     </row>
     <row r="29">
@@ -1076,13 +1076,13 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>1053576</v>
+        <v>1053575</v>
       </c>
       <c r="D31" t="n">
-        <v>1665015</v>
+        <v>1664904</v>
       </c>
       <c r="E31" t="n">
-        <v>611439</v>
+        <v>611329</v>
       </c>
     </row>
     <row r="32">
@@ -1181,13 +1181,13 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>496610</v>
+        <v>496576</v>
       </c>
       <c r="D36" t="n">
-        <v>818466</v>
+        <v>815791</v>
       </c>
       <c r="E36" t="n">
-        <v>321856</v>
+        <v>319215</v>
       </c>
     </row>
     <row r="37">
@@ -1223,13 +1223,13 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>343106</v>
+        <v>343103</v>
       </c>
       <c r="D38" t="n">
-        <v>523833</v>
+        <v>523500</v>
       </c>
       <c r="E38" t="n">
-        <v>180727</v>
+        <v>180397</v>
       </c>
     </row>
     <row r="39">
@@ -1244,13 +1244,13 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>413694</v>
+        <v>413690</v>
       </c>
       <c r="D39" t="n">
-        <v>635921</v>
+        <v>635477</v>
       </c>
       <c r="E39" t="n">
-        <v>222227</v>
+        <v>221787</v>
       </c>
     </row>
     <row r="40">
@@ -1307,13 +1307,13 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>181885</v>
+        <v>181884</v>
       </c>
       <c r="D42" t="n">
-        <v>282023</v>
+        <v>281912</v>
       </c>
       <c r="E42" t="n">
-        <v>100138</v>
+        <v>100028</v>
       </c>
     </row>
     <row r="43">
@@ -1370,13 +1370,13 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>236367</v>
+        <v>236363</v>
       </c>
       <c r="D45" t="n">
-        <v>377290</v>
+        <v>376846</v>
       </c>
       <c r="E45" t="n">
-        <v>140923</v>
+        <v>140483</v>
       </c>
     </row>
     <row r="46">
@@ -1412,13 +1412,13 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>191842</v>
+        <v>191841</v>
       </c>
       <c r="D47" t="n">
-        <v>303283</v>
+        <v>303172</v>
       </c>
       <c r="E47" t="n">
-        <v>111441</v>
+        <v>111331</v>
       </c>
     </row>
     <row r="48">
@@ -1454,13 +1454,13 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>364508</v>
+        <v>364505</v>
       </c>
       <c r="D49" t="n">
-        <v>575624</v>
+        <v>575291</v>
       </c>
       <c r="E49" t="n">
-        <v>211116</v>
+        <v>210786</v>
       </c>
     </row>
     <row r="50">
@@ -1538,13 +1538,13 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>180204</v>
+        <v>180203</v>
       </c>
       <c r="D53" t="n">
-        <v>277718</v>
+        <v>277607</v>
       </c>
       <c r="E53" t="n">
-        <v>97514</v>
+        <v>97404</v>
       </c>
     </row>
     <row r="54">
@@ -1559,13 +1559,13 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>360481</v>
+        <v>360478</v>
       </c>
       <c r="D54" t="n">
-        <v>570750</v>
+        <v>570417</v>
       </c>
       <c r="E54" t="n">
-        <v>210269</v>
+        <v>209939</v>
       </c>
     </row>
     <row r="55">
@@ -1685,13 +1685,13 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>244447</v>
+        <v>244446</v>
       </c>
       <c r="D60" t="n">
-        <v>375276</v>
+        <v>375165</v>
       </c>
       <c r="E60" t="n">
-        <v>130829</v>
+        <v>130719</v>
       </c>
     </row>
     <row r="61">
@@ -1727,13 +1727,13 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>188928</v>
+        <v>188927</v>
       </c>
       <c r="D62" t="n">
-        <v>287862</v>
+        <v>287751</v>
       </c>
       <c r="E62" t="n">
-        <v>98934</v>
+        <v>98824</v>
       </c>
     </row>
     <row r="63">
@@ -1769,13 +1769,13 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>106854</v>
+        <v>106853</v>
       </c>
       <c r="D64" t="n">
-        <v>166926</v>
+        <v>166815</v>
       </c>
       <c r="E64" t="n">
-        <v>60072</v>
+        <v>59962</v>
       </c>
     </row>
     <row r="65">
@@ -1790,13 +1790,13 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>85578</v>
+        <v>85577</v>
       </c>
       <c r="D65" t="n">
-        <v>128504</v>
+        <v>128393</v>
       </c>
       <c r="E65" t="n">
-        <v>42926</v>
+        <v>42816</v>
       </c>
     </row>
     <row r="66">
@@ -1895,13 +1895,13 @@
         </is>
       </c>
       <c r="C70" t="n">
-        <v>377184</v>
+        <v>377181</v>
       </c>
       <c r="D70" t="n">
-        <v>619650</v>
+        <v>619317</v>
       </c>
       <c r="E70" t="n">
-        <v>242466</v>
+        <v>242136</v>
       </c>
     </row>
     <row r="71">
@@ -2000,13 +2000,13 @@
         </is>
       </c>
       <c r="C75" t="n">
-        <v>102214</v>
+        <v>102213</v>
       </c>
       <c r="D75" t="n">
-        <v>156456</v>
+        <v>156345</v>
       </c>
       <c r="E75" t="n">
-        <v>54242</v>
+        <v>54132</v>
       </c>
     </row>
     <row r="76">
@@ -2063,13 +2063,13 @@
         </is>
       </c>
       <c r="C78" t="n">
-        <v>124148</v>
+        <v>124146</v>
       </c>
       <c r="D78" t="n">
-        <v>196271</v>
+        <v>196049</v>
       </c>
       <c r="E78" t="n">
-        <v>72123</v>
+        <v>71903</v>
       </c>
     </row>
     <row r="79">
@@ -2105,13 +2105,13 @@
         </is>
       </c>
       <c r="C80" t="n">
-        <v>824052</v>
+        <v>824049</v>
       </c>
       <c r="D80" t="n">
-        <v>1342430</v>
+        <v>1342097</v>
       </c>
       <c r="E80" t="n">
-        <v>518378</v>
+        <v>518048</v>
       </c>
     </row>
     <row r="81">
@@ -2126,13 +2126,13 @@
         </is>
       </c>
       <c r="C81" t="n">
-        <v>1823934</v>
+        <v>1823932</v>
       </c>
       <c r="D81" t="n">
-        <v>2916081</v>
+        <v>2915859</v>
       </c>
       <c r="E81" t="n">
-        <v>1092147</v>
+        <v>1091927</v>
       </c>
     </row>
     <row r="82">
@@ -2231,13 +2231,13 @@
         </is>
       </c>
       <c r="C86" t="n">
-        <v>1055770</v>
+        <v>1055769</v>
       </c>
       <c r="D86" t="n">
-        <v>1673992</v>
+        <v>1673881</v>
       </c>
       <c r="E86" t="n">
-        <v>618222</v>
+        <v>618112</v>
       </c>
     </row>
     <row r="87">
@@ -2399,13 +2399,13 @@
         </is>
       </c>
       <c r="C94" t="n">
-        <v>153278</v>
+        <v>153274</v>
       </c>
       <c r="D94" t="n">
-        <v>236193</v>
+        <v>235749</v>
       </c>
       <c r="E94" t="n">
-        <v>82915</v>
+        <v>82475</v>
       </c>
     </row>
     <row r="95">
@@ -2441,13 +2441,13 @@
         </is>
       </c>
       <c r="C96" t="n">
-        <v>244353</v>
+        <v>244351</v>
       </c>
       <c r="D96" t="n">
-        <v>382173</v>
+        <v>381951</v>
       </c>
       <c r="E96" t="n">
-        <v>137820</v>
+        <v>137600</v>
       </c>
     </row>
     <row r="97">
@@ -2462,13 +2462,13 @@
         </is>
       </c>
       <c r="C97" t="n">
-        <v>557340</v>
+        <v>557335</v>
       </c>
       <c r="D97" t="n">
-        <v>871332</v>
+        <v>870777</v>
       </c>
       <c r="E97" t="n">
-        <v>313992</v>
+        <v>313442</v>
       </c>
     </row>
     <row r="98">
@@ -2483,13 +2483,13 @@
         </is>
       </c>
       <c r="C98" t="n">
-        <v>273996</v>
+        <v>273993</v>
       </c>
       <c r="D98" t="n">
-        <v>455592</v>
+        <v>455259</v>
       </c>
       <c r="E98" t="n">
-        <v>181596</v>
+        <v>181266</v>
       </c>
     </row>
     <row r="99">
@@ -2504,13 +2504,13 @@
         </is>
       </c>
       <c r="C99" t="n">
-        <v>537425</v>
+        <v>537380</v>
       </c>
       <c r="D99" t="n">
-        <v>869436</v>
+        <v>864234</v>
       </c>
       <c r="E99" t="n">
-        <v>332011</v>
+        <v>326854</v>
       </c>
     </row>
     <row r="100">
@@ -2546,13 +2546,13 @@
         </is>
       </c>
       <c r="C101" t="n">
-        <v>495283</v>
+        <v>495277</v>
       </c>
       <c r="D101" t="n">
-        <v>765360</v>
+        <v>764694</v>
       </c>
       <c r="E101" t="n">
-        <v>270077</v>
+        <v>269417</v>
       </c>
     </row>
     <row r="102">
@@ -2567,13 +2567,13 @@
         </is>
       </c>
       <c r="C102" t="n">
-        <v>387551</v>
+        <v>387549</v>
       </c>
       <c r="D102" t="n">
-        <v>608808</v>
+        <v>608586</v>
       </c>
       <c r="E102" t="n">
-        <v>221257</v>
+        <v>221037</v>
       </c>
     </row>
     <row r="103">
@@ -2609,13 +2609,13 @@
         </is>
       </c>
       <c r="C104" t="n">
-        <v>253805</v>
+        <v>253803</v>
       </c>
       <c r="D104" t="n">
-        <v>399473</v>
+        <v>399251</v>
       </c>
       <c r="E104" t="n">
-        <v>145668</v>
+        <v>145448</v>
       </c>
     </row>
     <row r="105">
@@ -2756,13 +2756,13 @@
         </is>
       </c>
       <c r="C111" t="n">
-        <v>391847</v>
+        <v>391846</v>
       </c>
       <c r="D111" t="n">
-        <v>631520</v>
+        <v>631409</v>
       </c>
       <c r="E111" t="n">
-        <v>239673</v>
+        <v>239563</v>
       </c>
     </row>
     <row r="112">
@@ -2819,13 +2819,13 @@
         </is>
       </c>
       <c r="C114" t="n">
-        <v>472754</v>
+        <v>472753</v>
       </c>
       <c r="D114" t="n">
-        <v>753055</v>
+        <v>752944</v>
       </c>
       <c r="E114" t="n">
-        <v>280301</v>
+        <v>280191</v>
       </c>
     </row>
     <row r="115">
@@ -2840,13 +2840,13 @@
         </is>
       </c>
       <c r="C115" t="n">
-        <v>399092</v>
+        <v>399087</v>
       </c>
       <c r="D115" t="n">
-        <v>645325</v>
+        <v>644770</v>
       </c>
       <c r="E115" t="n">
-        <v>246233</v>
+        <v>245683</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update Design and add starts with and ends with in search
</commit_message>
<xml_diff>
--- a/verification_summary.xlsx
+++ b/verification_summary.xlsx
@@ -2504,13 +2504,13 @@
         </is>
       </c>
       <c r="C99" t="n">
-        <v>537367</v>
+        <v>537331</v>
       </c>
       <c r="D99" t="n">
-        <v>863890</v>
+        <v>863153</v>
       </c>
       <c r="E99" t="n">
-        <v>326523</v>
+        <v>325822</v>
       </c>
     </row>
     <row r="100">
@@ -2798,13 +2798,13 @@
         </is>
       </c>
       <c r="C113" t="n">
-        <v>535679</v>
+        <v>535680</v>
       </c>
       <c r="D113" t="n">
-        <v>858285</v>
+        <v>858396</v>
       </c>
       <c r="E113" t="n">
-        <v>322606</v>
+        <v>322716</v>
       </c>
     </row>
     <row r="114">

</xml_diff>

<commit_message>
surah yusuf aya 50
</commit_message>
<xml_diff>
--- a/verification_summary.xlsx
+++ b/verification_summary.xlsx
@@ -1076,13 +1076,13 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>1053560</v>
+        <v>1053559</v>
       </c>
       <c r="D31" t="n">
-        <v>1663239</v>
+        <v>1663128</v>
       </c>
       <c r="E31" t="n">
-        <v>609679</v>
+        <v>609569</v>
       </c>
     </row>
     <row r="32">
@@ -1181,13 +1181,13 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>496575</v>
+        <v>496882</v>
       </c>
       <c r="D36" t="n">
-        <v>815680</v>
+        <v>807205</v>
       </c>
       <c r="E36" t="n">
-        <v>319105</v>
+        <v>310323</v>
       </c>
     </row>
     <row r="37">
@@ -1202,13 +1202,13 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>179659</v>
+        <v>179658</v>
       </c>
       <c r="D37" t="n">
-        <v>303936</v>
+        <v>303825</v>
       </c>
       <c r="E37" t="n">
-        <v>124277</v>
+        <v>124167</v>
       </c>
     </row>
     <row r="38">
@@ -1223,13 +1223,13 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>343103</v>
+        <v>343102</v>
       </c>
       <c r="D38" t="n">
-        <v>523500</v>
+        <v>523389</v>
       </c>
       <c r="E38" t="n">
-        <v>180397</v>
+        <v>180287</v>
       </c>
     </row>
     <row r="39">
@@ -1286,13 +1286,13 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>70490</v>
+        <v>70489</v>
       </c>
       <c r="D41" t="n">
-        <v>107786</v>
+        <v>107675</v>
       </c>
       <c r="E41" t="n">
-        <v>37296</v>
+        <v>37186</v>
       </c>
     </row>
     <row r="42">
@@ -1496,13 +1496,13 @@
         </is>
       </c>
       <c r="C51" t="n">
-        <v>238765</v>
+        <v>238764</v>
       </c>
       <c r="D51" t="n">
-        <v>381844</v>
+        <v>381733</v>
       </c>
       <c r="E51" t="n">
-        <v>143079</v>
+        <v>142969</v>
       </c>
     </row>
     <row r="52">
@@ -2525,13 +2525,13 @@
         </is>
       </c>
       <c r="C100" t="n">
-        <v>334206</v>
+        <v>334205</v>
       </c>
       <c r="D100" t="n">
-        <v>532827</v>
+        <v>532716</v>
       </c>
       <c r="E100" t="n">
-        <v>198621</v>
+        <v>198511</v>
       </c>
     </row>
     <row r="101">
@@ -2546,13 +2546,13 @@
         </is>
       </c>
       <c r="C101" t="n">
-        <v>495277</v>
+        <v>495276</v>
       </c>
       <c r="D101" t="n">
-        <v>764694</v>
+        <v>764583</v>
       </c>
       <c r="E101" t="n">
-        <v>269417</v>
+        <v>269307</v>
       </c>
     </row>
     <row r="102">
@@ -2819,13 +2819,13 @@
         </is>
       </c>
       <c r="C114" t="n">
-        <v>472753</v>
+        <v>472752</v>
       </c>
       <c r="D114" t="n">
-        <v>752944</v>
+        <v>752833</v>
       </c>
       <c r="E114" t="n">
-        <v>280191</v>
+        <v>280081</v>
       </c>
     </row>
     <row r="115">

</xml_diff>

<commit_message>
surah yusuf aya 82 correction
</commit_message>
<xml_diff>
--- a/verification_summary.xlsx
+++ b/verification_summary.xlsx
@@ -1181,13 +1181,13 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>496882</v>
+        <v>496881</v>
       </c>
       <c r="D36" t="n">
-        <v>807205</v>
+        <v>807094</v>
       </c>
       <c r="E36" t="n">
-        <v>310323</v>
+        <v>310213</v>
       </c>
     </row>
     <row r="37">

</xml_diff>